<commit_message>
feat: Add TP réseau project, fix Notion logo, and improve E5 grid layout
</commit_message>
<xml_diff>
--- a/public/assets/grille.xlsx
+++ b/public/assets/grille.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kamdi\Desktop\PortfolioBTS\portfolio\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97705728-96D7-4237-A6E4-B73B79B865A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{419E7652-59C2-483C-940C-459D911F0A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$36</definedName>
   </definedNames>
   <calcPr calcId="101716"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="54">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -118,9 +118,6 @@
     <t>Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
-    <t>Adresse URL du portfolio :</t>
-  </si>
-  <si>
     <t>SESSION 2025</t>
   </si>
   <si>
@@ -197,6 +194,21 @@
   </si>
   <si>
     <t>Centre de formation : Lycée Frédéric Chopin</t>
+  </si>
+  <si>
+    <t>Test d'intégration du DashBoard SSO ( Stage 1er année)</t>
+  </si>
+  <si>
+    <t>Gestion droit d'accès TP SISR</t>
+  </si>
+  <si>
+    <t>Recensement et standards TP  SISR</t>
+  </si>
+  <si>
+    <t>Continuité et Surveillance TP SISR</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio : https://kamdine.netlify.app/#intro</t>
   </si>
 </sst>
 </file>
@@ -206,7 +218,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -273,6 +285,11 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="22"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -679,7 +696,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -747,77 +764,80 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1128,7 +1148,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ81"/>
+  <dimension ref="A1:AQ82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
@@ -1139,83 +1159,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="23"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
     </row>
     <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="30" t="s">
+      <c r="A3" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="25"/>
-      <c r="H3" s="31"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="47"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="27" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="29"/>
+      <c r="A4" s="43" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="44"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="45"/>
       <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
       <c r="G4" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="47" t="s">
+      <c r="H4" s="25" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="44"/>
+      <c r="A5" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="39"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="35" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1238,8 +1258,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="33"/>
-      <c r="B7" s="41"/>
+      <c r="A7" s="27"/>
+      <c r="B7" s="36"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1295,16 +1315,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="31"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1343,21 +1363,21 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B9" s="10">
         <v>2024</v>
       </c>
       <c r="C9" s="16"/>
-      <c r="D9" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="E9" s="46"/>
-      <c r="F9" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="G9" s="46" t="s">
-        <v>44</v>
+      <c r="D9" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="24" t="s">
+        <v>43</v>
       </c>
       <c r="H9" s="18"/>
       <c r="I9"/>
@@ -1398,21 +1418,21 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="10">
         <v>2025</v>
       </c>
       <c r="C10" s="17"/>
-      <c r="D10" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="E10" s="46"/>
-      <c r="F10" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="G10" s="46" t="s">
-        <v>44</v>
+      <c r="D10" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" s="24" t="s">
+        <v>43</v>
       </c>
       <c r="H10" s="18"/>
       <c r="I10"/>
@@ -1453,18 +1473,20 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B11" s="10">
         <v>2025</v>
       </c>
       <c r="C11" s="17"/>
-      <c r="D11" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="E11" s="46"/>
-      <c r="F11" s="46" t="s">
-        <v>44</v>
+      <c r="D11" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="24" t="s">
+        <v>43</v>
       </c>
       <c r="G11" s="17"/>
       <c r="H11" s="18"/>
@@ -1506,18 +1528,18 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B12" s="10">
         <v>2026</v>
       </c>
       <c r="C12" s="17"/>
-      <c r="D12" s="46" t="s">
-        <v>44</v>
+      <c r="D12" s="24" t="s">
+        <v>43</v>
       </c>
       <c r="E12" s="17"/>
-      <c r="F12" s="46" t="s">
-        <v>44</v>
+      <c r="F12" s="24" t="s">
+        <v>43</v>
       </c>
       <c r="G12" s="17"/>
       <c r="H12" s="18"/>
@@ -1559,7 +1581,7 @@
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B13" s="10">
         <v>2026</v>
@@ -1569,12 +1591,12 @@
       <c r="E13" s="17"/>
       <c r="F13" s="17"/>
       <c r="G13" s="17"/>
-      <c r="H13" s="46" t="s">
-        <v>44</v>
+      <c r="H13" s="24" t="s">
+        <v>43</v>
       </c>
       <c r="I13"/>
-      <c r="J13" s="45" t="s">
-        <v>29</v>
+      <c r="J13" s="23" t="s">
+        <v>28</v>
       </c>
       <c r="K13"/>
       <c r="L13"/>
@@ -1612,7 +1634,7 @@
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B14" s="10">
         <v>2026</v>
@@ -1622,8 +1644,8 @@
       <c r="E14" s="17"/>
       <c r="F14" s="17"/>
       <c r="G14" s="17"/>
-      <c r="H14" s="46" t="s">
-        <v>44</v>
+      <c r="H14" s="24" t="s">
+        <v>43</v>
       </c>
       <c r="I14"/>
       <c r="J14"/>
@@ -1663,13 +1685,13 @@
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B15" s="10">
         <v>2026</v>
       </c>
-      <c r="C15" s="46" t="s">
-        <v>44</v>
+      <c r="C15" s="24" t="s">
+        <v>43</v>
       </c>
       <c r="D15" s="17"/>
       <c r="E15" s="17"/>
@@ -1714,17 +1736,17 @@
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B16" s="10">
         <v>2024</v>
       </c>
-      <c r="C16" s="46" t="s">
-        <v>44</v>
-      </c>
+      <c r="C16" s="24"/>
       <c r="D16" s="17"/>
       <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
+      <c r="F16" s="48" t="s">
+        <v>43</v>
+      </c>
       <c r="G16" s="17"/>
       <c r="H16" s="18"/>
       <c r="I16"/>
@@ -1764,13 +1786,21 @@
       <c r="AQ16"/>
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="11"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="17"/>
+      <c r="A17" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="10">
+        <v>2026</v>
+      </c>
+      <c r="C17" s="48" t="s">
+        <v>43</v>
+      </c>
       <c r="D17" s="17"/>
       <c r="E17" s="17"/>
       <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
+      <c r="G17" s="48" t="s">
+        <v>43</v>
+      </c>
       <c r="H17" s="18"/>
       <c r="I17"/>
       <c r="J17"/>
@@ -1809,13 +1839,19 @@
       <c r="AQ17"/>
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="11"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="17"/>
+      <c r="A18" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="10">
+        <v>2026</v>
+      </c>
+      <c r="C18" s="48" t="s">
+        <v>43</v>
+      </c>
       <c r="D18" s="17"/>
       <c r="E18" s="17"/>
       <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
+      <c r="G18" s="48"/>
       <c r="H18" s="18"/>
       <c r="I18"/>
       <c r="J18"/>
@@ -1853,17 +1889,21 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="37" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="39"/>
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="10">
+        <v>2026</v>
+      </c>
+      <c r="C19" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="18"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1900,23 +1940,17 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="10">
-        <v>2025</v>
-      </c>
-      <c r="C20" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="D20" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="18"/>
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A20" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="34"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1955,16 +1989,14 @@
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B21" s="10">
         <v>2025</v>
       </c>
-      <c r="C21" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="D21" s="46" t="s">
-        <v>44</v>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24" t="s">
+        <v>43</v>
       </c>
       <c r="E21" s="17"/>
       <c r="F21" s="17"/>
@@ -2008,18 +2040,16 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B22" s="10">
         <v>2025</v>
       </c>
-      <c r="C22" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="E22" s="46"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E22" s="17"/>
       <c r="F22" s="17"/>
       <c r="G22" s="17"/>
       <c r="H22" s="18"/>
@@ -2061,20 +2091,18 @@
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B23" s="10">
         <v>2025</v>
       </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="E23" s="46" t="s">
-        <v>44</v>
-      </c>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E23" s="24"/>
       <c r="F23" s="17"/>
-      <c r="G23" s="46"/>
+      <c r="G23" s="17"/>
       <c r="H23" s="18"/>
       <c r="I23"/>
       <c r="J23"/>
@@ -2114,18 +2142,20 @@
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B24" s="10">
         <v>2025</v>
       </c>
       <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="G24" s="17"/>
+      <c r="D24" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E24" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="F24" s="17"/>
+      <c r="G24" s="24"/>
       <c r="H24" s="18"/>
       <c r="I24"/>
       <c r="J24"/>
@@ -2165,7 +2195,7 @@
     </row>
     <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="B25" s="10">
         <v>2025</v>
@@ -2173,11 +2203,11 @@
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
       <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
+      <c r="F25" s="24" t="s">
+        <v>43</v>
+      </c>
       <c r="G25" s="17"/>
-      <c r="H25" s="46" t="s">
-        <v>44</v>
-      </c>
+      <c r="H25" s="18"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2215,14 +2245,20 @@
       <c r="AQ25"/>
     </row>
     <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="11"/>
-      <c r="B26" s="10"/>
+      <c r="A26" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" s="10">
+        <v>2025</v>
+      </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
       <c r="E26" s="17"/>
       <c r="F26" s="17"/>
       <c r="G26" s="17"/>
-      <c r="H26" s="18"/>
+      <c r="H26" s="24" t="s">
+        <v>43</v>
+      </c>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2259,17 +2295,21 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="37" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" s="38"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="39"/>
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" s="10">
+        <v>2025</v>
+      </c>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="H27" s="18"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2306,21 +2346,17 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B28" s="10">
-        <v>2026</v>
-      </c>
-      <c r="C28" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="18"/>
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A28" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="B28" s="33"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="34"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2359,15 +2395,15 @@
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B29" s="10">
         <v>2026</v>
       </c>
-      <c r="C29" s="17"/>
-      <c r="D29" s="46" t="s">
-        <v>44</v>
-      </c>
+      <c r="C29" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" s="17"/>
       <c r="E29" s="17"/>
       <c r="F29" s="17"/>
       <c r="G29" s="17"/>
@@ -2410,19 +2446,19 @@
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B30" s="10">
         <v>2026</v>
       </c>
       <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
+      <c r="D30" s="24" t="s">
+        <v>43</v>
+      </c>
       <c r="E30" s="17"/>
       <c r="F30" s="17"/>
       <c r="G30" s="17"/>
-      <c r="H30" s="46" t="s">
-        <v>44</v>
-      </c>
+      <c r="H30" s="18"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2461,19 +2497,19 @@
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B31" s="10">
         <v>2026</v>
       </c>
       <c r="C31" s="17"/>
-      <c r="D31" s="46" t="s">
-        <v>44</v>
-      </c>
+      <c r="D31" s="17"/>
       <c r="E31" s="17"/>
       <c r="F31" s="17"/>
       <c r="G31" s="17"/>
-      <c r="H31" s="18"/>
+      <c r="H31" s="24" t="s">
+        <v>43</v>
+      </c>
       <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
@@ -2512,14 +2548,14 @@
     </row>
     <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B32" s="10">
         <v>2026</v>
       </c>
       <c r="C32" s="17"/>
-      <c r="D32" s="46" t="s">
-        <v>44</v>
+      <c r="D32" s="24" t="s">
+        <v>43</v>
       </c>
       <c r="E32" s="17"/>
       <c r="F32" s="17"/>
@@ -2562,20 +2598,20 @@
       <c r="AQ32"/>
     </row>
     <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="12" t="s">
-        <v>42</v>
+      <c r="A33" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="B33" s="10">
         <v>2026</v>
       </c>
-      <c r="C33" s="19"/>
-      <c r="D33" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="20"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+      <c r="H33" s="18"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2612,23 +2648,21 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="13" t="s">
-        <v>43</v>
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="B34" s="10">
         <v>2026</v>
       </c>
-      <c r="C34" s="21"/>
-      <c r="D34" s="21"/>
-      <c r="E34" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="F34" s="21"/>
-      <c r="G34" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="H34" s="22"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E34" s="19"/>
+      <c r="F34" s="19"/>
+      <c r="G34" s="19"/>
+      <c r="H34" s="20"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
@@ -2665,15 +2699,23 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A35" s="5"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
+    <row r="35" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35" s="10">
+        <v>2026</v>
+      </c>
+      <c r="C35" s="21"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="F35" s="21"/>
+      <c r="G35" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="H35" s="22"/>
       <c r="I35"/>
       <c r="J35"/>
       <c r="K35"/>
@@ -2710,7 +2752,51 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="36" spans="1:43" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A36" s="5"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4"/>
+      <c r="I36"/>
+      <c r="J36"/>
+      <c r="K36"/>
+      <c r="L36"/>
+      <c r="M36"/>
+      <c r="N36"/>
+      <c r="O36"/>
+      <c r="P36"/>
+      <c r="Q36"/>
+      <c r="R36"/>
+      <c r="S36"/>
+      <c r="T36"/>
+      <c r="U36"/>
+      <c r="V36"/>
+      <c r="W36"/>
+      <c r="X36"/>
+      <c r="Y36"/>
+      <c r="Z36"/>
+      <c r="AA36"/>
+      <c r="AB36"/>
+      <c r="AC36"/>
+      <c r="AD36"/>
+      <c r="AE36"/>
+      <c r="AF36"/>
+      <c r="AG36"/>
+      <c r="AH36"/>
+      <c r="AI36"/>
+      <c r="AJ36"/>
+      <c r="AK36"/>
+      <c r="AL36"/>
+      <c r="AM36"/>
+      <c r="AN36"/>
+      <c r="AO36"/>
+      <c r="AP36"/>
+      <c r="AQ36"/>
+    </row>
     <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -2756,20 +2842,21 @@
     <row r="79" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="80" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="81" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="82" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A5:H5"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="F3:H3"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A5:H5"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>